<commit_message>
Update of FWS metiers in Baltic
</commit_message>
<xml_diff>
--- a/Metiers/Reference_lists/RDB_ISSG_Metier_list.xlsx
+++ b/Metiers/Reference_lists/RDB_ISSG_Metier_list.xlsx
@@ -8292,7 +8292,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="189">
+  <cellXfs count="184">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -8576,9 +8576,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
@@ -8587,9 +8584,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="21" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -8616,15 +8610,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -8635,25 +8635,10 @@
     <xf numFmtId="1" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="0" fillId="21" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -8946,7 +8931,7 @@
     <col min="3" max="3" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="81.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="99.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="35.44140625" customWidth="1"/>
     <col min="7" max="7" width="13.33203125" style="82" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="106.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.21875" bestFit="1" customWidth="1"/>
@@ -9589,7 +9574,7 @@
         <v>1822</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9609,7 +9594,7 @@
         <v>1822</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9629,137 +9614,132 @@
         <v>1871</v>
       </c>
     </row>
-    <row r="35" spans="1:12" s="139" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="151" t="s">
+    <row r="35" spans="1:11" s="139" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="150" t="s">
         <v>1152</v>
       </c>
-      <c r="B35" s="152" t="s">
+      <c r="B35" s="151" t="s">
         <v>2177</v>
       </c>
       <c r="C35" s="149"/>
       <c r="D35" s="149"/>
       <c r="E35" s="149"/>
       <c r="F35" s="149"/>
-      <c r="G35" s="153"/>
-      <c r="H35" s="150" t="s">
+      <c r="G35" s="152" t="s">
         <v>1577</v>
       </c>
-      <c r="I35" s="149" t="s">
+      <c r="H35" s="96" t="s">
         <v>1871</v>
       </c>
-      <c r="J35" s="149"/>
-      <c r="K35" s="149">
+      <c r="I35" s="149"/>
+      <c r="J35" s="149">
         <v>20260422</v>
       </c>
-      <c r="L35" s="149" t="s">
+      <c r="K35" s="149" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="36" spans="1:12" s="139" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="151" t="s">
+    <row r="36" spans="1:11" s="139" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="150" t="s">
         <v>1152</v>
       </c>
-      <c r="B36" s="152" t="s">
+      <c r="B36" s="151" t="s">
         <v>2172</v>
       </c>
       <c r="C36" s="149"/>
       <c r="D36" s="149"/>
       <c r="E36" s="149"/>
       <c r="F36" s="149"/>
-      <c r="G36" s="153"/>
-      <c r="H36" s="150" t="s">
+      <c r="G36" s="181" t="s">
         <v>1577</v>
       </c>
-      <c r="I36" s="149" t="s">
+      <c r="H36" s="96" t="s">
         <v>1871</v>
       </c>
-      <c r="J36" s="149"/>
-      <c r="K36" s="149">
+      <c r="I36" s="149"/>
+      <c r="J36" s="149">
         <v>20260422</v>
       </c>
-      <c r="L36" s="149" t="s">
+      <c r="K36" s="149" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="37" spans="1:12" s="139" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="151" t="s">
+    <row r="37" spans="1:11" s="139" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="150" t="s">
         <v>1152</v>
       </c>
-      <c r="B37" s="152" t="s">
+      <c r="B37" s="151" t="s">
         <v>2174</v>
       </c>
       <c r="C37" s="149"/>
       <c r="D37" s="149"/>
       <c r="E37" s="149"/>
       <c r="F37" s="149"/>
-      <c r="G37" s="153"/>
-      <c r="H37" s="150" t="s">
+      <c r="G37" s="181" t="s">
         <v>1577</v>
       </c>
-      <c r="I37" s="149" t="s">
+      <c r="H37" s="96" t="s">
         <v>1871</v>
       </c>
-      <c r="J37" s="149"/>
-      <c r="K37" s="149">
+      <c r="I37" s="149"/>
+      <c r="J37" s="149">
         <v>20260422</v>
       </c>
-      <c r="L37" s="149" t="s">
+      <c r="K37" s="149" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="38" spans="1:12" s="139" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="151" t="s">
+    <row r="38" spans="1:11" s="139" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="150" t="s">
         <v>1152</v>
       </c>
-      <c r="B38" s="152" t="s">
+      <c r="B38" s="151" t="s">
         <v>2175</v>
       </c>
       <c r="C38" s="149"/>
       <c r="D38" s="149"/>
       <c r="E38" s="149"/>
       <c r="F38" s="149"/>
-      <c r="G38" s="153"/>
-      <c r="H38" s="150" t="s">
+      <c r="G38" s="181" t="s">
         <v>1577</v>
       </c>
-      <c r="I38" s="149" t="s">
+      <c r="H38" s="96" t="s">
         <v>1871</v>
       </c>
-      <c r="J38" s="149"/>
-      <c r="K38" s="149">
+      <c r="I38" s="149"/>
+      <c r="J38" s="149">
         <v>20260422</v>
       </c>
-      <c r="L38" s="149" t="s">
+      <c r="K38" s="149" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="39" spans="1:12" s="139" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="151" t="s">
+    <row r="39" spans="1:11" s="139" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="150" t="s">
         <v>1152</v>
       </c>
-      <c r="B39" s="152" t="s">
+      <c r="B39" s="151" t="s">
         <v>2176</v>
       </c>
       <c r="C39" s="149"/>
       <c r="D39" s="149"/>
       <c r="E39" s="149"/>
       <c r="F39" s="149"/>
-      <c r="G39" s="153"/>
-      <c r="H39" s="150" t="s">
+      <c r="G39" s="181" t="s">
         <v>1577</v>
       </c>
-      <c r="I39" s="149" t="s">
+      <c r="H39" s="96" t="s">
         <v>1871</v>
       </c>
-      <c r="J39" s="149"/>
-      <c r="K39" s="149">
+      <c r="I39" s="149"/>
+      <c r="J39" s="149">
         <v>20260422</v>
       </c>
-      <c r="L39" s="149" t="s">
+      <c r="K39" s="149" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9779,7 +9759,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9793,7 +9773,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9813,7 +9793,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9827,7 +9807,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9847,7 +9827,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9861,7 +9841,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9881,7 +9861,7 @@
         <v>1788</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>1152</v>
       </c>
@@ -9901,7 +9881,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" s="11" t="s">
         <v>1152</v>
       </c>
@@ -9923,7 +9903,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" s="11" t="s">
         <v>1152</v>
       </c>
@@ -9945,7 +9925,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" s="11" t="s">
         <v>1152</v>
       </c>
@@ -9967,7 +9947,7 @@
         <v>1823</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" s="11" t="s">
         <v>1152</v>
       </c>
@@ -9989,137 +9969,132 @@
         <v>1872</v>
       </c>
     </row>
-    <row r="52" spans="1:12" s="148" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="159" t="s">
+    <row r="52" spans="1:11" s="148" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="157" t="s">
         <v>1152</v>
       </c>
-      <c r="B52" s="157" t="s">
+      <c r="B52" s="155" t="s">
         <v>2182</v>
       </c>
-      <c r="C52" s="160"/>
-      <c r="D52" s="161"/>
-      <c r="E52" s="161"/>
-      <c r="F52" s="161"/>
-      <c r="G52" s="158"/>
-      <c r="H52" s="156" t="s">
+      <c r="C52" s="158"/>
+      <c r="D52" s="159"/>
+      <c r="E52" s="159"/>
+      <c r="F52" s="159"/>
+      <c r="G52" s="156" t="s">
         <v>1581</v>
       </c>
-      <c r="I52" s="155" t="s">
+      <c r="H52" s="96" t="s">
         <v>1872</v>
       </c>
-      <c r="J52" s="155"/>
-      <c r="K52" s="155">
+      <c r="I52" s="154"/>
+      <c r="J52" s="154">
         <v>20260422</v>
       </c>
-      <c r="L52" s="155" t="s">
+      <c r="K52" s="154" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="53" spans="1:12" s="148" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="159" t="s">
+    <row r="53" spans="1:11" s="148" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="157" t="s">
         <v>1152</v>
       </c>
-      <c r="B53" s="157" t="s">
+      <c r="B53" s="155" t="s">
         <v>2178</v>
       </c>
-      <c r="C53" s="160"/>
-      <c r="D53" s="161"/>
-      <c r="E53" s="161"/>
-      <c r="F53" s="161"/>
-      <c r="G53" s="158"/>
-      <c r="H53" s="156" t="s">
+      <c r="C53" s="158"/>
+      <c r="D53" s="159"/>
+      <c r="E53" s="159"/>
+      <c r="F53" s="159"/>
+      <c r="G53" s="165" t="s">
         <v>1581</v>
       </c>
-      <c r="I53" s="155" t="s">
+      <c r="H53" s="96" t="s">
         <v>1872</v>
       </c>
-      <c r="J53" s="155"/>
-      <c r="K53" s="155">
+      <c r="I53" s="154"/>
+      <c r="J53" s="154">
         <v>20260422</v>
       </c>
-      <c r="L53" s="155" t="s">
+      <c r="K53" s="154" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="54" spans="1:12" s="148" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="159" t="s">
+    <row r="54" spans="1:11" s="148" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="157" t="s">
         <v>1152</v>
       </c>
-      <c r="B54" s="157" t="s">
+      <c r="B54" s="155" t="s">
         <v>2179</v>
       </c>
-      <c r="C54" s="160"/>
-      <c r="D54" s="161"/>
-      <c r="E54" s="161"/>
-      <c r="F54" s="161"/>
-      <c r="G54" s="158"/>
-      <c r="H54" s="156" t="s">
+      <c r="C54" s="158"/>
+      <c r="D54" s="159"/>
+      <c r="E54" s="159"/>
+      <c r="F54" s="159"/>
+      <c r="G54" s="165" t="s">
         <v>1581</v>
       </c>
-      <c r="I54" s="155" t="s">
+      <c r="H54" s="96" t="s">
         <v>1872</v>
       </c>
-      <c r="J54" s="155"/>
-      <c r="K54" s="155">
+      <c r="I54" s="154"/>
+      <c r="J54" s="154">
         <v>20260422</v>
       </c>
-      <c r="L54" s="155" t="s">
+      <c r="K54" s="154" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="55" spans="1:12" s="148" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="159" t="s">
+    <row r="55" spans="1:11" s="148" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="157" t="s">
         <v>1152</v>
       </c>
-      <c r="B55" s="157" t="s">
+      <c r="B55" s="155" t="s">
         <v>2180</v>
       </c>
-      <c r="C55" s="160"/>
-      <c r="D55" s="161"/>
-      <c r="E55" s="161"/>
-      <c r="F55" s="161"/>
-      <c r="G55" s="158"/>
-      <c r="H55" s="156" t="s">
+      <c r="C55" s="158"/>
+      <c r="D55" s="159"/>
+      <c r="E55" s="159"/>
+      <c r="F55" s="159"/>
+      <c r="G55" s="165" t="s">
         <v>1581</v>
       </c>
-      <c r="I55" s="155" t="s">
+      <c r="H55" s="96" t="s">
         <v>1872</v>
       </c>
-      <c r="J55" s="155"/>
-      <c r="K55" s="155">
+      <c r="I55" s="154"/>
+      <c r="J55" s="154">
         <v>20260422</v>
       </c>
-      <c r="L55" s="155" t="s">
+      <c r="K55" s="154" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="56" spans="1:12" s="148" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="159" t="s">
+    <row r="56" spans="1:11" s="148" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="157" t="s">
         <v>1152</v>
       </c>
-      <c r="B56" s="157" t="s">
+      <c r="B56" s="155" t="s">
         <v>2181</v>
       </c>
-      <c r="C56" s="160"/>
-      <c r="D56" s="161"/>
-      <c r="E56" s="161"/>
-      <c r="F56" s="161"/>
-      <c r="G56" s="158"/>
-      <c r="H56" s="156" t="s">
+      <c r="C56" s="158"/>
+      <c r="D56" s="159"/>
+      <c r="E56" s="159"/>
+      <c r="F56" s="159"/>
+      <c r="G56" s="165" t="s">
         <v>1581</v>
       </c>
-      <c r="I56" s="155" t="s">
+      <c r="H56" s="96" t="s">
         <v>1872</v>
       </c>
-      <c r="J56" s="155"/>
-      <c r="K56" s="155">
+      <c r="I56" s="154"/>
+      <c r="J56" s="154">
         <v>20260422</v>
       </c>
-      <c r="L56" s="155" t="s">
+      <c r="K56" s="154" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10137,7 +10112,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10155,7 +10130,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10173,7 +10148,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10191,7 +10166,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10213,7 +10188,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>1152</v>
       </c>
@@ -10227,7 +10202,7 @@
         <v>1925</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>1152</v>
       </c>
@@ -10241,7 +10216,7 @@
         <v>1824</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>1152</v>
       </c>
@@ -10539,7 +10514,7 @@
         <v>1879</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A81" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10553,7 +10528,7 @@
         <v>1897</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10567,7 +10542,7 @@
         <v>1928</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10590,7 +10565,7 @@
         <v>1958</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A84" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10613,7 +10588,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A85" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10636,7 +10611,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A86" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10653,7 +10628,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A87" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10680,7 +10655,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A88" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10707,7 +10682,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A89" s="11" t="s">
         <v>1152</v>
       </c>
@@ -10731,7 +10706,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>1152</v>
       </c>
@@ -10752,7 +10727,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>1152</v>
       </c>
@@ -10773,7 +10748,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>1152</v>
       </c>
@@ -10794,7 +10769,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>1152</v>
       </c>
@@ -10819,7 +10794,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>1152</v>
       </c>
@@ -10844,203 +10819,196 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="95" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="165" t="s">
+    <row r="95" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="163" t="s">
         <v>1152</v>
       </c>
-      <c r="B95" s="166" t="s">
+      <c r="B95" s="164" t="s">
         <v>2183</v>
       </c>
-      <c r="C95" s="168"/>
-      <c r="D95" s="169"/>
-      <c r="E95" s="169"/>
-      <c r="F95" s="169"/>
-      <c r="G95" s="167"/>
-      <c r="H95" s="164" t="s">
+      <c r="C95" s="166"/>
+      <c r="D95" s="167"/>
+      <c r="E95" s="167"/>
+      <c r="F95" s="167"/>
+      <c r="G95" s="162" t="s">
         <v>1605</v>
       </c>
-      <c r="I95" s="163" t="s">
+      <c r="H95" s="161" t="s">
         <v>1875</v>
       </c>
-      <c r="J95" s="163" t="s">
+      <c r="I95" s="161" t="s">
         <v>1966</v>
       </c>
-      <c r="K95" s="163">
+      <c r="J95" s="161">
         <v>20260422</v>
       </c>
-      <c r="L95" s="163" t="s">
+      <c r="K95" s="161" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="96" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="165" t="s">
+    <row r="96" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="163" t="s">
         <v>1152</v>
       </c>
-      <c r="B96" s="166" t="s">
+      <c r="B96" s="164" t="s">
         <v>2184</v>
       </c>
-      <c r="C96" s="168"/>
-      <c r="D96" s="169"/>
-      <c r="E96" s="169"/>
-      <c r="F96" s="169"/>
-      <c r="G96" s="167"/>
-      <c r="H96" s="164" t="s">
+      <c r="C96" s="166"/>
+      <c r="D96" s="167"/>
+      <c r="E96" s="167"/>
+      <c r="F96" s="167"/>
+      <c r="G96" s="162" t="s">
         <v>1605</v>
       </c>
-      <c r="I96" s="163" t="s">
+      <c r="H96" s="161" t="s">
         <v>1875</v>
       </c>
-      <c r="J96" s="163" t="s">
+      <c r="I96" s="161" t="s">
         <v>1966</v>
       </c>
-      <c r="K96" s="163">
+      <c r="J96" s="161">
         <v>20260422</v>
       </c>
-      <c r="L96" s="163" t="s">
+      <c r="K96" s="161" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="97" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="165" t="s">
+    <row r="97" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="163" t="s">
         <v>1152</v>
       </c>
-      <c r="B97" s="166" t="s">
+      <c r="B97" s="164" t="s">
         <v>2185</v>
       </c>
-      <c r="C97" s="168"/>
-      <c r="D97" s="169"/>
-      <c r="E97" s="169"/>
-      <c r="F97" s="169"/>
-      <c r="G97" s="167"/>
-      <c r="H97" s="164" t="s">
+      <c r="C97" s="166"/>
+      <c r="D97" s="167"/>
+      <c r="E97" s="167"/>
+      <c r="F97" s="167"/>
+      <c r="G97" s="162" t="s">
         <v>1605</v>
       </c>
-      <c r="I97" s="163" t="s">
+      <c r="H97" s="161" t="s">
         <v>1875</v>
       </c>
-      <c r="J97" s="163" t="s">
+      <c r="I97" s="161" t="s">
         <v>1966</v>
       </c>
-      <c r="K97" s="163">
+      <c r="J97" s="161">
         <v>20260422</v>
       </c>
-      <c r="L97" s="163" t="s">
+      <c r="K97" s="161" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="98" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="165" t="s">
+    <row r="98" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="163" t="s">
         <v>1152</v>
       </c>
-      <c r="B98" s="166" t="s">
+      <c r="B98" s="164" t="s">
         <v>2186</v>
       </c>
-      <c r="C98" s="168"/>
-      <c r="D98" s="169"/>
-      <c r="E98" s="169"/>
-      <c r="F98" s="169"/>
-      <c r="G98" s="167"/>
-      <c r="H98" s="164" t="s">
+      <c r="C98" s="166"/>
+      <c r="D98" s="167"/>
+      <c r="E98" s="167"/>
+      <c r="F98" s="167"/>
+      <c r="G98" s="162" t="s">
         <v>1605</v>
       </c>
-      <c r="I98" s="163" t="s">
+      <c r="H98" s="161" t="s">
         <v>1875</v>
       </c>
-      <c r="J98" s="163" t="s">
+      <c r="I98" s="161" t="s">
         <v>1966</v>
       </c>
-      <c r="K98" s="163">
+      <c r="J98" s="161">
         <v>20260422</v>
       </c>
-      <c r="L98" s="163" t="s">
+      <c r="K98" s="161" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="99" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="165" t="s">
+    <row r="99" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="163" t="s">
         <v>1152</v>
       </c>
-      <c r="B99" s="166" t="s">
+      <c r="B99" s="164" t="s">
         <v>2187</v>
       </c>
-      <c r="C99" s="168"/>
-      <c r="D99" s="169"/>
-      <c r="E99" s="169"/>
-      <c r="F99" s="169"/>
-      <c r="G99" s="167"/>
-      <c r="H99" s="164" t="s">
+      <c r="C99" s="166"/>
+      <c r="D99" s="167"/>
+      <c r="E99" s="167"/>
+      <c r="F99" s="167"/>
+      <c r="G99" s="162" t="s">
         <v>1605</v>
       </c>
-      <c r="I99" s="163" t="s">
+      <c r="H99" s="161" t="s">
         <v>1875</v>
       </c>
-      <c r="J99" s="163" t="s">
+      <c r="I99" s="161" t="s">
         <v>1966</v>
       </c>
-      <c r="K99" s="163">
+      <c r="J99" s="161">
         <v>20260422</v>
       </c>
-      <c r="L99" s="163" t="s">
+      <c r="K99" s="161" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="100" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="165" t="s">
+    <row r="100" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="163" t="s">
         <v>1152</v>
       </c>
-      <c r="B100" s="166" t="s">
+      <c r="B100" s="164" t="s">
         <v>2188</v>
       </c>
-      <c r="C100" s="168"/>
-      <c r="D100" s="169"/>
-      <c r="E100" s="169"/>
-      <c r="F100" s="169"/>
-      <c r="G100" s="167"/>
-      <c r="H100" s="164" t="s">
+      <c r="C100" s="166"/>
+      <c r="D100" s="167"/>
+      <c r="E100" s="167"/>
+      <c r="F100" s="167"/>
+      <c r="G100" s="162" t="s">
         <v>1605</v>
       </c>
-      <c r="I100" s="163" t="s">
+      <c r="H100" s="161" t="s">
         <v>1875</v>
       </c>
-      <c r="J100" s="163" t="s">
+      <c r="I100" s="161" t="s">
         <v>1966</v>
       </c>
-      <c r="K100" s="163">
+      <c r="J100" s="161">
         <v>20260422</v>
       </c>
-      <c r="L100" s="163" t="s">
+      <c r="K100" s="161" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="101" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="165" t="s">
+    <row r="101" spans="1:11" s="153" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="163" t="s">
         <v>1152</v>
       </c>
-      <c r="B101" s="166" t="s">
+      <c r="B101" s="164" t="s">
         <v>2189</v>
       </c>
-      <c r="C101" s="168"/>
-      <c r="D101" s="169"/>
-      <c r="E101" s="169"/>
-      <c r="F101" s="169"/>
-      <c r="G101" s="167"/>
-      <c r="H101" s="164" t="s">
+      <c r="C101" s="166"/>
+      <c r="D101" s="167"/>
+      <c r="E101" s="167"/>
+      <c r="F101" s="167"/>
+      <c r="G101" s="162" t="s">
         <v>1605</v>
       </c>
-      <c r="I101" s="163" t="s">
+      <c r="H101" s="161" t="s">
         <v>1875</v>
       </c>
-      <c r="J101" s="163" t="s">
+      <c r="I101" s="161" t="s">
         <v>1966</v>
       </c>
-      <c r="K101" s="163">
+      <c r="J101" s="161">
         <v>20260422</v>
       </c>
-      <c r="L101" s="163" t="s">
+      <c r="K101" s="161" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11051,7 +11019,7 @@
       <c r="D102" s="3"/>
       <c r="E102" s="3"/>
       <c r="F102" s="3"/>
-      <c r="G102" s="81" t="s">
+      <c r="G102" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H102" t="s">
@@ -11064,7 +11032,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11075,7 +11043,7 @@
       <c r="D103" s="3"/>
       <c r="E103" s="3"/>
       <c r="F103" s="3"/>
-      <c r="G103" s="81" t="s">
+      <c r="G103" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H103" t="s">
@@ -11088,7 +11056,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11099,7 +11067,7 @@
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
       <c r="F104" s="3"/>
-      <c r="G104" s="81" t="s">
+      <c r="G104" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H104" t="s">
@@ -11112,7 +11080,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11125,7 +11093,7 @@
       </c>
       <c r="E105" s="3"/>
       <c r="F105" s="3"/>
-      <c r="G105" s="81" t="s">
+      <c r="G105" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H105" t="s">
@@ -11138,7 +11106,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11151,7 +11119,7 @@
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
       <c r="F106" s="3"/>
-      <c r="G106" s="81" t="s">
+      <c r="G106" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H106" t="s">
@@ -11164,7 +11132,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11175,7 +11143,7 @@
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
       <c r="F107" s="3"/>
-      <c r="G107" s="81" t="s">
+      <c r="G107" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H107" t="s">
@@ -11188,7 +11156,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11199,7 +11167,7 @@
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
       <c r="F108" s="3"/>
-      <c r="G108" s="81" t="s">
+      <c r="G108" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H108" t="s">
@@ -11212,7 +11180,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11223,7 +11191,7 @@
       <c r="D109" s="3"/>
       <c r="E109" s="3"/>
       <c r="F109" s="3"/>
-      <c r="G109" s="81" t="s">
+      <c r="G109" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H109" t="s">
@@ -11236,7 +11204,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11247,7 +11215,7 @@
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
       <c r="F110" s="3"/>
-      <c r="G110" s="81" t="s">
+      <c r="G110" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H110" t="s">
@@ -11260,7 +11228,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11271,7 +11239,7 @@
       <c r="D111" s="3"/>
       <c r="E111" s="3"/>
       <c r="F111" s="3"/>
-      <c r="G111" s="81" t="s">
+      <c r="G111" s="82" t="s">
         <v>1984</v>
       </c>
       <c r="H111" t="s">
@@ -11284,7 +11252,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11295,7 +11263,7 @@
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
       <c r="F112" s="3"/>
-      <c r="G112" s="81" t="s">
+      <c r="G112" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H112" t="s">
@@ -11320,7 +11288,7 @@
       <c r="F113" s="3" t="s">
         <v>534</v>
       </c>
-      <c r="G113" s="81" t="s">
+      <c r="G113" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H113" t="s">
@@ -11337,7 +11305,7 @@
       <c r="B114" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="G114" s="81" t="s">
+      <c r="G114" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H114" t="s">
@@ -11357,7 +11325,7 @@
       <c r="D115">
         <v>2010</v>
       </c>
-      <c r="G115" s="81" t="s">
+      <c r="G115" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H115" t="s">
@@ -11383,7 +11351,7 @@
       <c r="F116" t="s">
         <v>455</v>
       </c>
-      <c r="G116" s="81" t="s">
+      <c r="G116" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H116" t="s">
@@ -11401,7 +11369,7 @@
         <v>2000</v>
       </c>
       <c r="E117" s="4"/>
-      <c r="G117" s="81" t="s">
+      <c r="G117" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H117" t="s">
@@ -11421,7 +11389,7 @@
       <c r="B118" s="22" t="s">
         <v>1172</v>
       </c>
-      <c r="G118" s="81" t="s">
+      <c r="G118" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H118" t="s">
@@ -11444,7 +11412,7 @@
       <c r="F119" t="s">
         <v>750</v>
       </c>
-      <c r="G119" s="81" t="s">
+      <c r="G119" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H119" t="s">
@@ -11467,7 +11435,7 @@
       <c r="F120" t="s">
         <v>718</v>
       </c>
-      <c r="G120" s="81" t="s">
+      <c r="G120" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H120" t="s">
@@ -11490,7 +11458,7 @@
       <c r="F121" t="s">
         <v>729</v>
       </c>
-      <c r="G121" s="81" t="s">
+      <c r="G121" s="82" t="s">
         <v>1606</v>
       </c>
       <c r="H121" t="s">
@@ -11513,7 +11481,7 @@
       <c r="F122" t="s">
         <v>743</v>
       </c>
-      <c r="G122" s="81" t="s">
+      <c r="G122" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H122" t="s">
@@ -11533,7 +11501,7 @@
       <c r="F123" t="s">
         <v>771</v>
       </c>
-      <c r="G123" s="81" t="s">
+      <c r="G123" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H123" t="s">
@@ -11547,7 +11515,7 @@
       <c r="B124" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="G124" s="81" t="s">
+      <c r="G124" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H124" t="s">
@@ -11570,7 +11538,7 @@
       <c r="F125" t="s">
         <v>774</v>
       </c>
-      <c r="G125" s="81" t="s">
+      <c r="G125" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H125" t="s">
@@ -11593,7 +11561,7 @@
       <c r="F126" t="s">
         <v>775</v>
       </c>
-      <c r="G126" s="81" t="s">
+      <c r="G126" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H126" t="s">
@@ -11608,7 +11576,7 @@
         <v>2001</v>
       </c>
       <c r="E127" s="4"/>
-      <c r="G127" s="81" t="s">
+      <c r="G127" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H127" t="s">
@@ -11626,42 +11594,42 @@
         <v>1176</v>
       </c>
       <c r="E128" s="4"/>
-      <c r="G128" s="81" t="s">
+      <c r="G128" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H128" t="s">
         <v>1829</v>
       </c>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B129" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="G129" s="81" t="s">
+      <c r="G129" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H129" t="s">
         <v>1829</v>
       </c>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B130" s="23" t="s">
         <v>660</v>
       </c>
-      <c r="G130" s="81" t="s">
+      <c r="G130" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H130" t="s">
         <v>1829</v>
       </c>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11674,14 +11642,14 @@
       <c r="F131" t="s">
         <v>752</v>
       </c>
-      <c r="G131" s="81" t="s">
+      <c r="G131" s="82" t="s">
         <v>1607</v>
       </c>
       <c r="H131" t="s">
         <v>1829</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11694,238 +11662,231 @@
       <c r="F132" t="s">
         <v>753</v>
       </c>
-      <c r="G132" s="81" t="s">
+      <c r="G132" s="82" t="s">
         <v>1608</v>
       </c>
       <c r="H132" t="s">
         <v>1876</v>
       </c>
     </row>
-    <row r="133" spans="1:12" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A133" s="173" t="s">
+    <row r="133" spans="1:11" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A133" s="170" t="s">
         <v>1152</v>
       </c>
-      <c r="B133" s="171" t="s">
+      <c r="B133" s="169" t="s">
         <v>2190</v>
       </c>
-      <c r="C133" s="171"/>
-      <c r="D133" s="171"/>
-      <c r="E133" s="171"/>
-      <c r="F133" s="171"/>
-      <c r="G133" s="174"/>
-      <c r="H133" s="172" t="s">
+      <c r="C133" s="169"/>
+      <c r="D133" s="169"/>
+      <c r="E133" s="169"/>
+      <c r="F133" s="169"/>
+      <c r="G133" s="183" t="s">
         <v>1608</v>
       </c>
-      <c r="I133" s="171" t="s">
+      <c r="H133" s="169" t="s">
         <v>1876</v>
       </c>
-      <c r="J133" s="171"/>
-      <c r="K133" s="171">
+      <c r="I133" s="169"/>
+      <c r="J133" s="178">
         <v>20260422</v>
       </c>
-      <c r="L133" s="171" t="s">
+      <c r="K133" s="169" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="134" spans="1:12" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A134" s="173" t="s">
+    <row r="134" spans="1:11" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A134" s="170" t="s">
         <v>1152</v>
       </c>
-      <c r="B134" s="171" t="s">
+      <c r="B134" s="169" t="s">
         <v>2191</v>
       </c>
-      <c r="C134" s="171"/>
-      <c r="D134" s="171"/>
-      <c r="E134" s="171"/>
-      <c r="F134" s="171"/>
-      <c r="G134" s="174"/>
-      <c r="H134" s="172" t="s">
+      <c r="C134" s="169"/>
+      <c r="D134" s="169"/>
+      <c r="E134" s="169"/>
+      <c r="F134" s="169"/>
+      <c r="G134" s="183" t="s">
         <v>1608</v>
       </c>
-      <c r="I134" s="171" t="s">
+      <c r="H134" s="169" t="s">
         <v>1876</v>
       </c>
-      <c r="J134" s="171"/>
-      <c r="K134" s="171">
+      <c r="I134" s="169"/>
+      <c r="J134" s="178">
         <v>20260422</v>
       </c>
-      <c r="L134" s="171" t="s">
+      <c r="K134" s="169" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="135" spans="1:12" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A135" s="173" t="s">
+    <row r="135" spans="1:11" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A135" s="170" t="s">
         <v>1152</v>
       </c>
-      <c r="B135" s="171" t="s">
+      <c r="B135" s="169" t="s">
         <v>2192</v>
       </c>
-      <c r="C135" s="171"/>
-      <c r="D135" s="171"/>
-      <c r="E135" s="171"/>
-      <c r="F135" s="171"/>
-      <c r="G135" s="174"/>
-      <c r="H135" s="172" t="s">
+      <c r="C135" s="169"/>
+      <c r="D135" s="169"/>
+      <c r="E135" s="169"/>
+      <c r="F135" s="169"/>
+      <c r="G135" s="183" t="s">
         <v>1608</v>
       </c>
-      <c r="I135" s="171" t="s">
+      <c r="H135" s="169" t="s">
         <v>1876</v>
       </c>
-      <c r="J135" s="171"/>
-      <c r="K135" s="171">
+      <c r="I135" s="169"/>
+      <c r="J135" s="178">
         <v>20260422</v>
       </c>
-      <c r="L135" s="171" t="s">
+      <c r="K135" s="169" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="136" spans="1:12" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A136" s="173" t="s">
+    <row r="136" spans="1:11" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A136" s="170" t="s">
         <v>1152</v>
       </c>
-      <c r="B136" s="171" t="s">
+      <c r="B136" s="169" t="s">
         <v>2193</v>
       </c>
-      <c r="C136" s="171"/>
-      <c r="D136" s="171"/>
-      <c r="E136" s="171"/>
-      <c r="F136" s="171"/>
-      <c r="G136" s="174"/>
-      <c r="H136" s="172" t="s">
+      <c r="C136" s="169"/>
+      <c r="D136" s="169"/>
+      <c r="E136" s="169"/>
+      <c r="F136" s="169"/>
+      <c r="G136" s="183" t="s">
         <v>1608</v>
       </c>
-      <c r="I136" s="171" t="s">
+      <c r="H136" s="169" t="s">
         <v>1876</v>
       </c>
-      <c r="J136" s="171"/>
-      <c r="K136" s="171">
+      <c r="I136" s="169"/>
+      <c r="J136" s="178">
         <v>20260422</v>
       </c>
-      <c r="L136" s="171" t="s">
+      <c r="K136" s="169" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="137" spans="1:12" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A137" s="173" t="s">
+    <row r="137" spans="1:11" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A137" s="170" t="s">
         <v>1152</v>
       </c>
-      <c r="B137" s="171" t="s">
+      <c r="B137" s="169" t="s">
         <v>2194</v>
       </c>
-      <c r="C137" s="171"/>
-      <c r="D137" s="171"/>
-      <c r="E137" s="171"/>
-      <c r="F137" s="171"/>
-      <c r="G137" s="174"/>
-      <c r="H137" s="172" t="s">
+      <c r="C137" s="169"/>
+      <c r="D137" s="169"/>
+      <c r="E137" s="169"/>
+      <c r="F137" s="169"/>
+      <c r="G137" s="183" t="s">
         <v>1608</v>
       </c>
-      <c r="I137" s="171" t="s">
+      <c r="H137" s="169" t="s">
         <v>1876</v>
       </c>
-      <c r="J137" s="171"/>
-      <c r="K137" s="171">
+      <c r="I137" s="169"/>
+      <c r="J137" s="178">
         <v>20260422</v>
       </c>
-      <c r="L137" s="171" t="s">
+      <c r="K137" s="169" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="138" spans="1:12" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A138" s="173" t="s">
+    <row r="138" spans="1:11" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="170" t="s">
         <v>1152</v>
       </c>
-      <c r="B138" s="171" t="s">
+      <c r="B138" s="169" t="s">
         <v>2195</v>
       </c>
-      <c r="C138" s="171"/>
-      <c r="D138" s="171"/>
-      <c r="E138" s="171"/>
-      <c r="F138" s="171"/>
-      <c r="G138" s="174"/>
-      <c r="H138" s="172" t="s">
+      <c r="C138" s="169"/>
+      <c r="D138" s="169"/>
+      <c r="E138" s="169"/>
+      <c r="F138" s="169"/>
+      <c r="G138" s="183" t="s">
         <v>1608</v>
       </c>
-      <c r="I138" s="171" t="s">
+      <c r="H138" s="169" t="s">
         <v>1876</v>
       </c>
-      <c r="J138" s="171"/>
-      <c r="K138" s="171">
+      <c r="I138" s="169"/>
+      <c r="J138" s="178">
         <v>20260422</v>
       </c>
-      <c r="L138" s="171" t="s">
+      <c r="K138" s="169" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="139" spans="1:12" s="162" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A139" s="173" t="s">
+    <row r="139" spans="1:11" s="160" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="170" t="s">
         <v>1152</v>
       </c>
-      <c r="B139" s="171" t="s">
+      <c r="B139" s="169" t="s">
         <v>2196</v>
       </c>
-      <c r="C139" s="171"/>
-      <c r="D139" s="171"/>
-      <c r="E139" s="171"/>
-      <c r="F139" s="171"/>
-      <c r="G139" s="174"/>
-      <c r="H139" s="172" t="s">
+      <c r="C139" s="169"/>
+      <c r="D139" s="169"/>
+      <c r="E139" s="169"/>
+      <c r="F139" s="169"/>
+      <c r="G139" s="183" t="s">
         <v>1608</v>
       </c>
-      <c r="I139" s="171" t="s">
+      <c r="H139" s="169" t="s">
         <v>1876</v>
       </c>
-      <c r="J139" s="171"/>
-      <c r="K139" s="171">
+      <c r="I139" s="169"/>
+      <c r="J139" s="178">
         <v>20260422</v>
       </c>
-      <c r="L139" s="171" t="s">
+      <c r="K139" s="169" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B140" s="9" t="s">
         <v>405</v>
       </c>
-      <c r="G140" s="81" t="s">
+      <c r="G140" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H140" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B141" s="9" t="s">
         <v>1182</v>
       </c>
-      <c r="G141" s="81" t="s">
+      <c r="G141" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H141" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B142" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="G142" s="81" t="s">
+      <c r="G142" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H142" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11941,14 +11902,14 @@
       <c r="F143" t="s">
         <v>455</v>
       </c>
-      <c r="G143" s="81" t="s">
+      <c r="G143" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H143" t="s">
         <v>1949</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>1152</v>
       </c>
@@ -11964,7 +11925,7 @@
       <c r="F144" t="s">
         <v>760</v>
       </c>
-      <c r="G144" s="81" t="s">
+      <c r="G144" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H144" t="s">
@@ -11979,7 +11940,7 @@
         <v>2002</v>
       </c>
       <c r="E145" s="4"/>
-      <c r="G145" s="81" t="s">
+      <c r="G145" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H145" t="s">
@@ -11996,7 +11957,7 @@
       <c r="B146" s="9" t="s">
         <v>1181</v>
       </c>
-      <c r="G146" s="81" t="s">
+      <c r="G146" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H146" t="s">
@@ -12016,7 +11977,7 @@
       <c r="F147" t="s">
         <v>731</v>
       </c>
-      <c r="G147" s="81" t="s">
+      <c r="G147" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H147" t="s">
@@ -12036,7 +11997,7 @@
       <c r="F148" t="s">
         <v>723</v>
       </c>
-      <c r="G148" s="81" t="s">
+      <c r="G148" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H148" t="s">
@@ -12050,7 +12011,7 @@
       <c r="B149" s="9" t="s">
         <v>663</v>
       </c>
-      <c r="G149" s="81" t="s">
+      <c r="G149" s="82" t="s">
         <v>1609</v>
       </c>
       <c r="H149" t="s">
@@ -12064,15 +12025,16 @@
       <c r="B150" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="G150" s="81" t="s">
+      <c r="G150" t="s">
         <v>1610</v>
       </c>
-      <c r="H150" t="s">
+      <c r="H150" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I150" t="s">
+      <c r="I150" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J150" s="175"/>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
@@ -12087,15 +12049,16 @@
       <c r="F151" t="s">
         <v>546</v>
       </c>
-      <c r="G151" s="81" t="s">
+      <c r="G151" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H151" t="s">
+      <c r="H151" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I151" t="s">
+      <c r="I151" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J151" s="175"/>
     </row>
     <row r="152" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
@@ -12104,15 +12067,16 @@
       <c r="B152" s="24" t="s">
         <v>131</v>
       </c>
-      <c r="G152" s="81" t="s">
+      <c r="G152" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H152" t="s">
+      <c r="H152" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I152" t="s">
+      <c r="I152" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J152" s="175"/>
     </row>
     <row r="153" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
@@ -12130,15 +12094,16 @@
       <c r="F153" t="s">
         <v>546</v>
       </c>
-      <c r="G153" s="81" t="s">
+      <c r="G153" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H153" t="s">
+      <c r="H153" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I153" t="s">
+      <c r="I153" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J153" s="175"/>
     </row>
     <row r="154" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
@@ -12156,15 +12121,16 @@
       <c r="F154" t="s">
         <v>740</v>
       </c>
-      <c r="G154" s="81" t="s">
+      <c r="G154" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H154" t="s">
+      <c r="H154" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I154" t="s">
+      <c r="I154" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J154" s="175"/>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
@@ -12174,16 +12140,16 @@
         <v>1974</v>
       </c>
       <c r="E155" s="4"/>
-      <c r="G155" s="81" t="s">
+      <c r="G155" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H155" t="s">
+      <c r="H155" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I155" t="s">
+      <c r="I155" s="175" t="s">
         <v>1966</v>
       </c>
-      <c r="J155">
+      <c r="J155" s="175">
         <v>20220909</v>
       </c>
     </row>
@@ -12195,15 +12161,16 @@
         <v>1185</v>
       </c>
       <c r="E156" s="4"/>
-      <c r="G156" s="81" t="s">
+      <c r="G156" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H156" t="s">
+      <c r="H156" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I156" t="s">
+      <c r="I156" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J156" s="175"/>
     </row>
     <row r="157" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
@@ -12212,15 +12179,16 @@
       <c r="B157" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="G157" s="81" t="s">
+      <c r="G157" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H157" t="s">
+      <c r="H157" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I157" t="s">
+      <c r="I157" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J157" s="175"/>
     </row>
     <row r="158" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
@@ -12229,15 +12197,16 @@
       <c r="B158" s="24" t="s">
         <v>665</v>
       </c>
-      <c r="G158" s="81" t="s">
+      <c r="G158" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H158" t="s">
+      <c r="H158" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I158" t="s">
+      <c r="I158" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J158" s="175"/>
     </row>
     <row r="159" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
@@ -12246,15 +12215,16 @@
       <c r="B159" s="24" t="s">
         <v>666</v>
       </c>
-      <c r="G159" s="81" t="s">
+      <c r="G159" s="175" t="s">
         <v>1610</v>
       </c>
-      <c r="H159" t="s">
+      <c r="H159" s="175" t="s">
         <v>1830</v>
       </c>
-      <c r="I159" t="s">
+      <c r="I159" s="175" t="s">
         <v>1966</v>
       </c>
+      <c r="J159" s="175"/>
     </row>
     <row r="160" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
@@ -12263,12 +12233,14 @@
       <c r="B160" s="23" t="s">
         <v>668</v>
       </c>
-      <c r="G160" s="81" t="s">
+      <c r="G160" t="s">
         <v>1703</v>
       </c>
-      <c r="H160" t="s">
+      <c r="H160" s="175" t="s">
         <v>1931</v>
       </c>
+      <c r="I160" s="175"/>
+      <c r="J160" s="175"/>
     </row>
     <row r="161" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
@@ -12277,12 +12249,14 @@
       <c r="B161" s="23" t="s">
         <v>1190</v>
       </c>
-      <c r="G161" s="81" t="s">
+      <c r="G161" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H161" t="s">
+      <c r="H161" s="175" t="s">
         <v>1931</v>
       </c>
+      <c r="I161" s="175"/>
+      <c r="J161" s="175"/>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
@@ -12291,12 +12265,14 @@
       <c r="B162" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="G162" s="81" t="s">
+      <c r="G162" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H162" t="s">
+      <c r="H162" s="175" t="s">
         <v>1931</v>
       </c>
+      <c r="I162" s="175"/>
+      <c r="J162" s="175"/>
     </row>
     <row r="163" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
@@ -12308,12 +12284,14 @@
       <c r="D163">
         <v>2010</v>
       </c>
-      <c r="G163" s="81" t="s">
+      <c r="G163" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H163" t="s">
+      <c r="H163" s="175" t="s">
         <v>1950</v>
       </c>
+      <c r="I163" s="175"/>
+      <c r="J163" s="175"/>
     </row>
     <row r="164" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
@@ -12325,12 +12303,14 @@
       <c r="C164">
         <v>2011</v>
       </c>
-      <c r="G164" s="81" t="s">
+      <c r="G164" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H164" t="s">
+      <c r="H164" s="175" t="s">
         <v>1946</v>
       </c>
+      <c r="I164" s="175"/>
+      <c r="J164" s="175"/>
     </row>
     <row r="165" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
@@ -12339,13 +12319,14 @@
       <c r="B165" s="23" t="s">
         <v>2003</v>
       </c>
-      <c r="G165" s="81" t="s">
+      <c r="G165" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H165" t="s">
+      <c r="H165" s="175" t="s">
         <v>1931</v>
       </c>
-      <c r="J165">
+      <c r="I165" s="175"/>
+      <c r="J165" s="175">
         <v>20220909</v>
       </c>
     </row>
@@ -12356,12 +12337,14 @@
       <c r="B166" s="23" t="s">
         <v>1189</v>
       </c>
-      <c r="G166" s="81" t="s">
+      <c r="G166" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H166" t="s">
+      <c r="H166" s="175" t="s">
         <v>1931</v>
       </c>
+      <c r="I166" s="175"/>
+      <c r="J166" s="175"/>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
@@ -12376,12 +12359,14 @@
       <c r="F167" t="s">
         <v>725</v>
       </c>
-      <c r="G167" s="81" t="s">
+      <c r="G167" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H167" t="s">
+      <c r="H167" s="175" t="s">
         <v>1931</v>
       </c>
+      <c r="I167" s="175"/>
+      <c r="J167" s="175"/>
     </row>
     <row r="168" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
@@ -12396,12 +12381,14 @@
       <c r="F168" t="s">
         <v>546</v>
       </c>
-      <c r="G168" s="81" t="s">
+      <c r="G168" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H168" t="s">
+      <c r="H168" s="175" t="s">
         <v>1931</v>
       </c>
+      <c r="I168" s="175"/>
+      <c r="J168" s="175"/>
     </row>
     <row r="169" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
@@ -12410,12 +12397,14 @@
       <c r="B169" s="23" t="s">
         <v>670</v>
       </c>
-      <c r="G169" s="81" t="s">
+      <c r="G169" s="175" t="s">
         <v>1703</v>
       </c>
-      <c r="H169" t="s">
+      <c r="H169" s="175" t="s">
         <v>1931</v>
       </c>
+      <c r="I169" s="175"/>
+      <c r="J169" s="175"/>
     </row>
     <row r="170" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
@@ -12430,7 +12419,7 @@
       <c r="F170" t="s">
         <v>455</v>
       </c>
-      <c r="G170" s="81" t="s">
+      <c r="G170" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H170" t="s">
@@ -12447,7 +12436,7 @@
       <c r="B171" s="25" t="s">
         <v>1194</v>
       </c>
-      <c r="G171" s="81" t="s">
+      <c r="G171" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H171" t="s">
@@ -12464,7 +12453,7 @@
       <c r="B172" s="25" t="s">
         <v>163</v>
       </c>
-      <c r="G172" s="81" t="s">
+      <c r="G172" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H172" t="s">
@@ -12490,7 +12479,7 @@
       <c r="F173" t="s">
         <v>531</v>
       </c>
-      <c r="G173" s="81" t="s">
+      <c r="G173" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H173" t="s">
@@ -12516,7 +12505,7 @@
       <c r="F174" t="s">
         <v>718</v>
       </c>
-      <c r="G174" s="81" t="s">
+      <c r="G174" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H174" t="s">
@@ -12534,7 +12523,7 @@
         <v>2004</v>
       </c>
       <c r="E175" s="4"/>
-      <c r="G175" s="81" t="s">
+      <c r="G175" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H175" t="s">
@@ -12554,7 +12543,7 @@
       <c r="B176" s="25" t="s">
         <v>1193</v>
       </c>
-      <c r="G176" s="81" t="s">
+      <c r="G176" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H176" t="s">
@@ -12564,14 +12553,14 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B177" s="25" t="s">
         <v>158</v>
       </c>
-      <c r="G177" s="81" t="s">
+      <c r="G177" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H177" t="s">
@@ -12581,14 +12570,14 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B178" s="25" t="s">
         <v>672</v>
       </c>
-      <c r="G178" s="81" t="s">
+      <c r="G178" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H178" t="s">
@@ -12598,7 +12587,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
         <v>1152</v>
       </c>
@@ -12611,7 +12600,7 @@
       <c r="F179" t="s">
         <v>563</v>
       </c>
-      <c r="G179" s="81" t="s">
+      <c r="G179" s="82" t="s">
         <v>1611</v>
       </c>
       <c r="H179" t="s">
@@ -12621,7 +12610,7 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
         <v>1152</v>
       </c>
@@ -12634,7 +12623,7 @@
       <c r="F180" t="s">
         <v>740</v>
       </c>
-      <c r="G180" s="81" t="s">
+      <c r="G180" s="82" t="s">
         <v>1612</v>
       </c>
       <c r="H180" t="s">
@@ -12644,210 +12633,203 @@
         <v>1966</v>
       </c>
     </row>
-    <row r="181" spans="1:12" s="170" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A181" s="178" t="s">
+    <row r="181" spans="1:11" s="168" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A181" s="174" t="s">
         <v>1152</v>
       </c>
-      <c r="B181" s="176" t="s">
+      <c r="B181" s="172" t="s">
         <v>2197</v>
       </c>
-      <c r="C181" s="176"/>
-      <c r="D181" s="176"/>
-      <c r="E181" s="176"/>
-      <c r="F181" s="176"/>
-      <c r="G181" s="179"/>
-      <c r="H181" s="177" t="s">
+      <c r="C181" s="172"/>
+      <c r="D181" s="172"/>
+      <c r="E181" s="172"/>
+      <c r="F181" s="172"/>
+      <c r="G181" s="173" t="s">
         <v>1612</v>
       </c>
-      <c r="I181" s="176" t="s">
+      <c r="H181" s="172" t="s">
         <v>1877</v>
       </c>
-      <c r="J181" s="176" t="s">
+      <c r="I181" s="172" t="s">
         <v>1966</v>
       </c>
-      <c r="K181" s="176">
+      <c r="J181" s="172">
         <v>20260422</v>
       </c>
-      <c r="L181" s="176" t="s">
+      <c r="K181" s="172" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="182" spans="1:12" s="170" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A182" s="178" t="s">
+    <row r="182" spans="1:11" s="168" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A182" s="174" t="s">
         <v>1152</v>
       </c>
-      <c r="B182" s="176" t="s">
+      <c r="B182" s="172" t="s">
         <v>2198</v>
       </c>
-      <c r="C182" s="176"/>
-      <c r="D182" s="176"/>
-      <c r="E182" s="176"/>
-      <c r="F182" s="176"/>
-      <c r="G182" s="179"/>
-      <c r="H182" s="177" t="s">
+      <c r="C182" s="172"/>
+      <c r="D182" s="172"/>
+      <c r="E182" s="172"/>
+      <c r="F182" s="172"/>
+      <c r="G182" s="173" t="s">
         <v>1612</v>
       </c>
-      <c r="I182" s="176" t="s">
+      <c r="H182" s="172" t="s">
         <v>1877</v>
       </c>
-      <c r="J182" s="176" t="s">
+      <c r="I182" s="172" t="s">
         <v>1966</v>
       </c>
-      <c r="K182" s="176">
+      <c r="J182" s="172">
         <v>20260422</v>
       </c>
-      <c r="L182" s="176" t="s">
+      <c r="K182" s="172" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="183" spans="1:12" s="170" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A183" s="178" t="s">
+    <row r="183" spans="1:11" s="168" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A183" s="174" t="s">
         <v>1152</v>
       </c>
-      <c r="B183" s="176" t="s">
+      <c r="B183" s="172" t="s">
         <v>2199</v>
       </c>
-      <c r="C183" s="176"/>
-      <c r="D183" s="176"/>
-      <c r="E183" s="176"/>
-      <c r="F183" s="176"/>
-      <c r="G183" s="179"/>
-      <c r="H183" s="177" t="s">
+      <c r="C183" s="172"/>
+      <c r="D183" s="172"/>
+      <c r="E183" s="172"/>
+      <c r="F183" s="172"/>
+      <c r="G183" s="173" t="s">
         <v>1612</v>
       </c>
-      <c r="I183" s="176" t="s">
+      <c r="H183" s="172" t="s">
         <v>1877</v>
       </c>
-      <c r="J183" s="176" t="s">
+      <c r="I183" s="172" t="s">
         <v>1966</v>
       </c>
-      <c r="K183" s="176">
+      <c r="J183" s="172">
         <v>20260422</v>
       </c>
-      <c r="L183" s="176" t="s">
+      <c r="K183" s="172" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="184" spans="1:12" s="170" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A184" s="178" t="s">
+    <row r="184" spans="1:11" s="168" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A184" s="174" t="s">
         <v>1152</v>
       </c>
-      <c r="B184" s="176" t="s">
+      <c r="B184" s="172" t="s">
         <v>2200</v>
       </c>
-      <c r="C184" s="176"/>
-      <c r="D184" s="176"/>
-      <c r="E184" s="176"/>
-      <c r="F184" s="176"/>
-      <c r="G184" s="179"/>
-      <c r="H184" s="177" t="s">
+      <c r="C184" s="172"/>
+      <c r="D184" s="172"/>
+      <c r="E184" s="172"/>
+      <c r="F184" s="172"/>
+      <c r="G184" s="173" t="s">
         <v>1612</v>
       </c>
-      <c r="I184" s="176" t="s">
+      <c r="H184" s="172" t="s">
         <v>1877</v>
       </c>
-      <c r="J184" s="176" t="s">
+      <c r="I184" s="172" t="s">
         <v>1966</v>
       </c>
-      <c r="K184" s="176">
+      <c r="J184" s="172">
         <v>20260422</v>
       </c>
-      <c r="L184" s="176" t="s">
+      <c r="K184" s="172" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="185" spans="1:12" s="170" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A185" s="178" t="s">
+    <row r="185" spans="1:11" s="168" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A185" s="174" t="s">
         <v>1152</v>
       </c>
-      <c r="B185" s="176" t="s">
+      <c r="B185" s="172" t="s">
         <v>2201</v>
       </c>
-      <c r="C185" s="176"/>
-      <c r="D185" s="176"/>
-      <c r="E185" s="176"/>
-      <c r="F185" s="176"/>
-      <c r="G185" s="179"/>
-      <c r="H185" s="177" t="s">
+      <c r="C185" s="172"/>
+      <c r="D185" s="172"/>
+      <c r="E185" s="172"/>
+      <c r="F185" s="172"/>
+      <c r="G185" s="173" t="s">
         <v>1612</v>
       </c>
-      <c r="I185" s="176" t="s">
+      <c r="H185" s="172" t="s">
         <v>1877</v>
       </c>
-      <c r="J185" s="176" t="s">
+      <c r="I185" s="172" t="s">
         <v>1966</v>
       </c>
-      <c r="K185" s="176">
+      <c r="J185" s="172">
         <v>20260422</v>
       </c>
-      <c r="L185" s="176" t="s">
+      <c r="K185" s="172" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="186" spans="1:12" s="170" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A186" s="178" t="s">
+    <row r="186" spans="1:11" s="168" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A186" s="174" t="s">
         <v>1152</v>
       </c>
-      <c r="B186" s="176" t="s">
+      <c r="B186" s="172" t="s">
         <v>2202</v>
       </c>
-      <c r="C186" s="176"/>
-      <c r="D186" s="176"/>
-      <c r="E186" s="176"/>
-      <c r="F186" s="176"/>
-      <c r="G186" s="179"/>
-      <c r="H186" s="177" t="s">
+      <c r="C186" s="172"/>
+      <c r="D186" s="172"/>
+      <c r="E186" s="172"/>
+      <c r="F186" s="172"/>
+      <c r="G186" s="173" t="s">
         <v>1612</v>
       </c>
-      <c r="I186" s="176" t="s">
+      <c r="H186" s="172" t="s">
         <v>1877</v>
       </c>
-      <c r="J186" s="176" t="s">
+      <c r="I186" s="172" t="s">
         <v>1966</v>
       </c>
-      <c r="K186" s="176">
+      <c r="J186" s="172">
         <v>20260422</v>
       </c>
-      <c r="L186" s="176" t="s">
+      <c r="K186" s="172" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="187" spans="1:12" s="170" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A187" s="178" t="s">
+    <row r="187" spans="1:11" s="168" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A187" s="174" t="s">
         <v>1152</v>
       </c>
-      <c r="B187" s="176" t="s">
+      <c r="B187" s="172" t="s">
         <v>2203</v>
       </c>
-      <c r="C187" s="176"/>
-      <c r="D187" s="176"/>
-      <c r="E187" s="176"/>
-      <c r="F187" s="176"/>
-      <c r="G187" s="179"/>
-      <c r="H187" s="177" t="s">
+      <c r="C187" s="172"/>
+      <c r="D187" s="172"/>
+      <c r="E187" s="172"/>
+      <c r="F187" s="172"/>
+      <c r="G187" s="173" t="s">
         <v>1612</v>
       </c>
-      <c r="I187" s="176" t="s">
+      <c r="H187" s="172" t="s">
         <v>1877</v>
       </c>
-      <c r="J187" s="176" t="s">
+      <c r="I187" s="172" t="s">
         <v>1966</v>
       </c>
-      <c r="K187" s="176">
+      <c r="J187" s="172">
         <v>20260422</v>
       </c>
-      <c r="L187" s="176" t="s">
+      <c r="K187" s="172" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B188" s="26" t="s">
         <v>371</v>
       </c>
-      <c r="G188" s="81" t="s">
+      <c r="G188" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H188" t="s">
@@ -12857,14 +12839,14 @@
         <v>1962</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A189" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B189" s="26" t="s">
         <v>1198</v>
       </c>
-      <c r="G189" s="81" t="s">
+      <c r="G189" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H189" t="s">
@@ -12874,14 +12856,14 @@
         <v>1962</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B190" s="26" t="s">
         <v>169</v>
       </c>
-      <c r="G190" s="81" t="s">
+      <c r="G190" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H190" t="s">
@@ -12891,7 +12873,7 @@
         <v>1962</v>
       </c>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A191" s="1" t="s">
         <v>1152</v>
       </c>
@@ -12907,7 +12889,7 @@
       <c r="F191" t="s">
         <v>455</v>
       </c>
-      <c r="G191" s="81" t="s">
+      <c r="G191" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H191" t="s">
@@ -12917,7 +12899,7 @@
         <v>1962</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>1152</v>
       </c>
@@ -12933,7 +12915,7 @@
       <c r="F192" t="s">
         <v>743</v>
       </c>
-      <c r="G192" s="81" t="s">
+      <c r="G192" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H192" t="s">
@@ -12951,7 +12933,7 @@
         <v>2005</v>
       </c>
       <c r="E193" s="4"/>
-      <c r="G193" s="81" t="s">
+      <c r="G193" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H193" t="s">
@@ -12971,7 +12953,7 @@
       <c r="B194" s="26" t="s">
         <v>1197</v>
       </c>
-      <c r="G194" s="81" t="s">
+      <c r="G194" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H194" t="s">
@@ -12994,7 +12976,7 @@
       <c r="F195" t="s">
         <v>718</v>
       </c>
-      <c r="G195" s="81" t="s">
+      <c r="G195" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H195" t="s">
@@ -13017,7 +12999,7 @@
       <c r="F196" t="s">
         <v>718</v>
       </c>
-      <c r="G196" s="81" t="s">
+      <c r="G196" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H196" t="s">
@@ -13034,7 +13016,7 @@
       <c r="B197" s="26" t="s">
         <v>675</v>
       </c>
-      <c r="G197" s="81" t="s">
+      <c r="G197" s="82" t="s">
         <v>1613</v>
       </c>
       <c r="H197" t="s">
@@ -13057,7 +13039,7 @@
       <c r="F198" t="s">
         <v>743</v>
       </c>
-      <c r="G198" s="81" t="s">
+      <c r="G198" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H198" t="s">
@@ -13071,7 +13053,7 @@
       <c r="B199" s="27" t="s">
         <v>1202</v>
       </c>
-      <c r="G199" s="81" t="s">
+      <c r="G199" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H199" t="s">
@@ -13085,7 +13067,7 @@
       <c r="B200" s="27" t="s">
         <v>176</v>
       </c>
-      <c r="G200" s="81" t="s">
+      <c r="G200" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H200" t="s">
@@ -13108,7 +13090,7 @@
       <c r="F201" t="s">
         <v>729</v>
       </c>
-      <c r="G201" s="81" t="s">
+      <c r="G201" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H201" t="s">
@@ -13131,7 +13113,7 @@
       <c r="F202" t="s">
         <v>748</v>
       </c>
-      <c r="G202" s="81" t="s">
+      <c r="G202" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H202" t="s">
@@ -13146,7 +13128,7 @@
         <v>2006</v>
       </c>
       <c r="E203" s="4"/>
-      <c r="G203" s="81" t="s">
+      <c r="G203" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H203" t="s">
@@ -13163,7 +13145,7 @@
       <c r="B204" s="27" t="s">
         <v>1201</v>
       </c>
-      <c r="G204" s="81" t="s">
+      <c r="G204" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H204" t="s">
@@ -13177,7 +13159,7 @@
       <c r="B205" s="27" t="s">
         <v>171</v>
       </c>
-      <c r="G205" s="81" t="s">
+      <c r="G205" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H205" t="s">
@@ -13191,7 +13173,7 @@
       <c r="B206" s="27" t="s">
         <v>678</v>
       </c>
-      <c r="G206" s="81" t="s">
+      <c r="G206" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H206" t="s">
@@ -13211,7 +13193,7 @@
       <c r="F207" t="s">
         <v>563</v>
       </c>
-      <c r="G207" s="81" t="s">
+      <c r="G207" s="82" t="s">
         <v>1614</v>
       </c>
       <c r="H207" t="s">
@@ -13231,196 +13213,189 @@
       <c r="F208" t="s">
         <v>759</v>
       </c>
-      <c r="G208" s="81" t="s">
+      <c r="G208" s="82" t="s">
         <v>1615</v>
       </c>
       <c r="H208" t="s">
         <v>1876</v>
       </c>
     </row>
-    <row r="209" spans="1:12" s="175" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A209" s="183" t="s">
+    <row r="209" spans="1:11" s="171" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A209" s="177" t="s">
         <v>1152</v>
       </c>
-      <c r="B209" s="181" t="s">
+      <c r="B209" s="176" t="s">
         <v>2204</v>
       </c>
-      <c r="C209" s="181"/>
-      <c r="D209" s="181"/>
-      <c r="E209" s="181"/>
-      <c r="F209" s="181"/>
-      <c r="G209" s="184"/>
-      <c r="H209" s="182" t="s">
+      <c r="C209" s="176"/>
+      <c r="D209" s="176"/>
+      <c r="E209" s="176"/>
+      <c r="F209" s="176"/>
+      <c r="G209" s="82" t="s">
         <v>1615</v>
       </c>
-      <c r="I209" s="181" t="s">
+      <c r="H209" s="178" t="s">
         <v>1876</v>
       </c>
-      <c r="J209" s="181"/>
-      <c r="K209" s="181">
+      <c r="I209" s="176"/>
+      <c r="J209" s="178">
         <v>20260422</v>
       </c>
-      <c r="L209" s="181" t="s">
+      <c r="K209" s="176" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="210" spans="1:12" s="175" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A210" s="183" t="s">
+    <row r="210" spans="1:11" s="171" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A210" s="177" t="s">
         <v>1152</v>
       </c>
-      <c r="B210" s="181" t="s">
+      <c r="B210" s="176" t="s">
         <v>2205</v>
       </c>
-      <c r="C210" s="181"/>
-      <c r="D210" s="181"/>
-      <c r="E210" s="181"/>
-      <c r="F210" s="181"/>
-      <c r="G210" s="184"/>
-      <c r="H210" s="182" t="s">
+      <c r="C210" s="176"/>
+      <c r="D210" s="176"/>
+      <c r="E210" s="176"/>
+      <c r="F210" s="176"/>
+      <c r="G210" s="82" t="s">
         <v>1615</v>
       </c>
-      <c r="I210" s="181" t="s">
+      <c r="H210" s="178" t="s">
         <v>1876</v>
       </c>
-      <c r="J210" s="181"/>
-      <c r="K210" s="181">
+      <c r="I210" s="176"/>
+      <c r="J210" s="178">
         <v>20260422</v>
       </c>
-      <c r="L210" s="181" t="s">
+      <c r="K210" s="176" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="211" spans="1:12" s="175" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A211" s="183" t="s">
+    <row r="211" spans="1:11" s="171" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A211" s="177" t="s">
         <v>1152</v>
       </c>
-      <c r="B211" s="181" t="s">
+      <c r="B211" s="176" t="s">
         <v>2206</v>
       </c>
-      <c r="C211" s="181"/>
-      <c r="D211" s="181"/>
-      <c r="E211" s="181"/>
-      <c r="F211" s="181"/>
-      <c r="G211" s="184"/>
-      <c r="H211" s="182" t="s">
+      <c r="C211" s="176"/>
+      <c r="D211" s="176"/>
+      <c r="E211" s="176"/>
+      <c r="F211" s="176"/>
+      <c r="G211" s="82" t="s">
         <v>1615</v>
       </c>
-      <c r="I211" s="181" t="s">
+      <c r="H211" s="178" t="s">
         <v>1876</v>
       </c>
-      <c r="J211" s="181"/>
-      <c r="K211" s="181">
+      <c r="I211" s="176"/>
+      <c r="J211" s="178">
         <v>20260422</v>
       </c>
-      <c r="L211" s="181" t="s">
+      <c r="K211" s="176" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="212" spans="1:12" s="175" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A212" s="183" t="s">
+    <row r="212" spans="1:11" s="171" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A212" s="177" t="s">
         <v>1152</v>
       </c>
-      <c r="B212" s="181" t="s">
+      <c r="B212" s="176" t="s">
         <v>2207</v>
       </c>
-      <c r="C212" s="181"/>
-      <c r="D212" s="181"/>
-      <c r="E212" s="181"/>
-      <c r="F212" s="181"/>
-      <c r="G212" s="184"/>
-      <c r="H212" s="182" t="s">
+      <c r="C212" s="176"/>
+      <c r="D212" s="176"/>
+      <c r="E212" s="176"/>
+      <c r="F212" s="176"/>
+      <c r="G212" s="82" t="s">
         <v>1615</v>
       </c>
-      <c r="I212" s="181" t="s">
+      <c r="H212" s="178" t="s">
         <v>1876</v>
       </c>
-      <c r="J212" s="181"/>
-      <c r="K212" s="181">
+      <c r="I212" s="176"/>
+      <c r="J212" s="178">
         <v>20260422</v>
       </c>
-      <c r="L212" s="181" t="s">
+      <c r="K212" s="176" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="213" spans="1:12" s="175" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A213" s="183" t="s">
+    <row r="213" spans="1:11" s="171" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A213" s="177" t="s">
         <v>1152</v>
       </c>
-      <c r="B213" s="181" t="s">
+      <c r="B213" s="176" t="s">
         <v>2208</v>
       </c>
-      <c r="C213" s="181"/>
-      <c r="D213" s="181"/>
-      <c r="E213" s="181"/>
-      <c r="F213" s="181"/>
-      <c r="G213" s="184"/>
-      <c r="H213" s="182" t="s">
+      <c r="C213" s="176"/>
+      <c r="D213" s="176"/>
+      <c r="E213" s="176"/>
+      <c r="F213" s="176"/>
+      <c r="G213" s="82" t="s">
         <v>1615</v>
       </c>
-      <c r="I213" s="181" t="s">
+      <c r="H213" s="178" t="s">
         <v>1876</v>
       </c>
-      <c r="J213" s="181"/>
-      <c r="K213" s="181">
+      <c r="I213" s="176"/>
+      <c r="J213" s="178">
         <v>20260422</v>
       </c>
-      <c r="L213" s="181" t="s">
+      <c r="K213" s="176" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="214" spans="1:12" s="175" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A214" s="183" t="s">
+    <row r="214" spans="1:11" s="171" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A214" s="177" t="s">
         <v>1152</v>
       </c>
-      <c r="B214" s="181" t="s">
+      <c r="B214" s="176" t="s">
         <v>2209</v>
       </c>
-      <c r="C214" s="181"/>
-      <c r="D214" s="181"/>
-      <c r="E214" s="181"/>
-      <c r="F214" s="181"/>
-      <c r="G214" s="184"/>
-      <c r="H214" s="182" t="s">
+      <c r="C214" s="176"/>
+      <c r="D214" s="176"/>
+      <c r="E214" s="176"/>
+      <c r="F214" s="176"/>
+      <c r="G214" s="82" t="s">
         <v>1615</v>
       </c>
-      <c r="I214" s="181" t="s">
+      <c r="H214" s="178" t="s">
         <v>1876</v>
       </c>
-      <c r="J214" s="181"/>
-      <c r="K214" s="181">
+      <c r="I214" s="176"/>
+      <c r="J214" s="178">
         <v>20260422</v>
       </c>
-      <c r="L214" s="181" t="s">
+      <c r="K214" s="176" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="215" spans="1:12" s="175" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A215" s="183" t="s">
+    <row r="215" spans="1:11" s="171" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A215" s="177" t="s">
         <v>1152</v>
       </c>
-      <c r="B215" s="181" t="s">
+      <c r="B215" s="176" t="s">
         <v>2210</v>
       </c>
-      <c r="C215" s="181"/>
-      <c r="D215" s="181"/>
-      <c r="E215" s="181"/>
-      <c r="F215" s="181"/>
-      <c r="G215" s="184"/>
-      <c r="H215" s="182" t="s">
+      <c r="C215" s="176"/>
+      <c r="D215" s="176"/>
+      <c r="E215" s="176"/>
+      <c r="F215" s="176"/>
+      <c r="G215" s="82" t="s">
         <v>1615</v>
       </c>
-      <c r="I215" s="181" t="s">
+      <c r="H215" s="178" t="s">
         <v>1876</v>
       </c>
-      <c r="J215" s="181"/>
-      <c r="K215" s="181">
+      <c r="I215" s="176"/>
+      <c r="J215" s="178">
         <v>20260422</v>
       </c>
-      <c r="L215" s="181" t="s">
+      <c r="K215" s="176" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A216" s="1" t="s">
         <v>1152</v>
       </c>
@@ -13433,42 +13408,42 @@
       <c r="F216" t="s">
         <v>760</v>
       </c>
-      <c r="G216" s="81" t="s">
+      <c r="G216" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H216" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A217" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B217" s="28" t="s">
         <v>1206</v>
       </c>
-      <c r="G217" s="81" t="s">
+      <c r="G217" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H217" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A218" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B218" s="28" t="s">
         <v>186</v>
       </c>
-      <c r="G218" s="81" t="s">
+      <c r="G218" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H218" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A219" s="1" t="s">
         <v>1152</v>
       </c>
@@ -13484,14 +13459,14 @@
       <c r="F219" t="s">
         <v>455</v>
       </c>
-      <c r="G219" s="81" t="s">
+      <c r="G219" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H219" t="s">
         <v>1949</v>
       </c>
     </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A220" s="1" t="s">
         <v>1152</v>
       </c>
@@ -13507,14 +13482,14 @@
       <c r="F220" t="s">
         <v>534</v>
       </c>
-      <c r="G220" s="81" t="s">
+      <c r="G220" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H220" t="s">
         <v>1945</v>
       </c>
     </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A221" s="1" t="s">
         <v>1152</v>
       </c>
@@ -13522,7 +13497,7 @@
         <v>2007</v>
       </c>
       <c r="E221" s="4"/>
-      <c r="G221" s="81" t="s">
+      <c r="G221" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H221" t="s">
@@ -13532,21 +13507,21 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="222" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A222" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B222" s="28" t="s">
         <v>1205</v>
       </c>
-      <c r="G222" s="81" t="s">
+      <c r="G222" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H222" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A223" s="11" t="s">
         <v>1152</v>
       </c>
@@ -13559,14 +13534,14 @@
       <c r="F223" t="s">
         <v>750</v>
       </c>
-      <c r="G223" s="81" t="s">
+      <c r="G223" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H223" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A224" s="11" t="s">
         <v>1152</v>
       </c>
@@ -13579,7 +13554,7 @@
       <c r="F224" t="s">
         <v>718</v>
       </c>
-      <c r="G224" s="81" t="s">
+      <c r="G224" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H224" t="s">
@@ -13599,7 +13574,7 @@
       <c r="F225" t="s">
         <v>729</v>
       </c>
-      <c r="G225" s="81" t="s">
+      <c r="G225" s="82" t="s">
         <v>1616</v>
       </c>
       <c r="H225" t="s">
@@ -13613,7 +13588,7 @@
       <c r="B226" s="29" t="s">
         <v>1154</v>
       </c>
-      <c r="G226" s="81" t="s">
+      <c r="G226" s="82" t="s">
         <v>1704</v>
       </c>
       <c r="H226" t="s">
@@ -13633,7 +13608,7 @@
       <c r="F227" t="s">
         <v>721</v>
       </c>
-      <c r="G227" s="81" t="s">
+      <c r="G227" s="82" t="s">
         <v>1705</v>
       </c>
       <c r="H227" t="s">
@@ -13647,7 +13622,7 @@
       <c r="B228" s="29" t="s">
         <v>188</v>
       </c>
-      <c r="G228" s="81" t="s">
+      <c r="G228" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H228" t="s">
@@ -13664,7 +13639,7 @@
       <c r="B229" s="29" t="s">
         <v>1210</v>
       </c>
-      <c r="G229" s="81" t="s">
+      <c r="G229" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H229" t="s">
@@ -13685,7 +13660,7 @@
       <c r="D230" s="3"/>
       <c r="E230" s="3"/>
       <c r="F230" s="3"/>
-      <c r="G230" s="81" t="s">
+      <c r="G230" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H230" t="s">
@@ -13712,7 +13687,7 @@
       <c r="F231" s="3" t="s">
         <v>772</v>
       </c>
-      <c r="G231" s="81" t="s">
+      <c r="G231" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H231" t="s">
@@ -13739,7 +13714,7 @@
       <c r="F232" s="3" t="s">
         <v>773</v>
       </c>
-      <c r="G232" s="81" t="s">
+      <c r="G232" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H232" t="s">
@@ -13760,7 +13735,7 @@
       <c r="D233" s="3"/>
       <c r="E233" s="76"/>
       <c r="F233" s="3"/>
-      <c r="G233" s="81" t="s">
+      <c r="G233" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H233" t="s">
@@ -13784,7 +13759,7 @@
       <c r="D234" s="3"/>
       <c r="E234" s="3"/>
       <c r="F234" s="3"/>
-      <c r="G234" s="81" t="s">
+      <c r="G234" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H234" t="s">
@@ -13803,7 +13778,7 @@
       </c>
       <c r="E235" s="3"/>
       <c r="F235" s="3"/>
-      <c r="G235" s="81" t="s">
+      <c r="G235" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H235" t="s">
@@ -13826,7 +13801,7 @@
       <c r="F236" s="3" t="s">
         <v>764</v>
       </c>
-      <c r="G236" s="81" t="s">
+      <c r="G236" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H236" t="s">
@@ -13849,7 +13824,7 @@
       <c r="F237" s="3" t="s">
         <v>729</v>
       </c>
-      <c r="G237" s="81" t="s">
+      <c r="G237" s="82" t="s">
         <v>1617</v>
       </c>
       <c r="H237" t="s">
@@ -13866,7 +13841,7 @@
       <c r="B238" s="27" t="s">
         <v>1322</v>
       </c>
-      <c r="G238" s="81" t="s">
+      <c r="G238" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H238" t="s">
@@ -13886,7 +13861,7 @@
       <c r="B239" s="27" t="s">
         <v>1986</v>
       </c>
-      <c r="G239" s="81" t="s">
+      <c r="G239" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H239" t="s">
@@ -13906,7 +13881,7 @@
       <c r="B240" s="27" t="s">
         <v>1331</v>
       </c>
-      <c r="G240" s="81" t="s">
+      <c r="G240" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H240" t="s">
@@ -13929,7 +13904,7 @@
       <c r="D241">
         <v>2010</v>
       </c>
-      <c r="G241" s="81" t="s">
+      <c r="G241" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H241" t="s">
@@ -13952,7 +13927,7 @@
       <c r="C242">
         <v>2011</v>
       </c>
-      <c r="G242" s="81" t="s">
+      <c r="G242" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H242" t="s">
@@ -13972,7 +13947,7 @@
       <c r="B243" s="27" t="s">
         <v>2009</v>
       </c>
-      <c r="G243" s="81" t="s">
+      <c r="G243" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H243" t="s">
@@ -13992,7 +13967,7 @@
       <c r="B244" s="27" t="s">
         <v>1989</v>
       </c>
-      <c r="G244" s="81" t="s">
+      <c r="G244" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H244" t="s">
@@ -14012,7 +13987,7 @@
       <c r="B245" s="27" t="s">
         <v>1323</v>
       </c>
-      <c r="G245" s="81" t="s">
+      <c r="G245" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H245" t="s">
@@ -14032,7 +14007,7 @@
       <c r="B246" s="27" t="s">
         <v>1990</v>
       </c>
-      <c r="G246" s="81" t="s">
+      <c r="G246" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H246" t="s">
@@ -14052,7 +14027,7 @@
       <c r="B247" s="27" t="s">
         <v>1991</v>
       </c>
-      <c r="G247" s="81" t="s">
+      <c r="G247" s="82" t="s">
         <v>1695</v>
       </c>
       <c r="H247" t="s">
@@ -14072,7 +14047,7 @@
       <c r="B248" s="27" t="s">
         <v>1726</v>
       </c>
-      <c r="G248" s="81" t="s">
+      <c r="G248" s="82" t="s">
         <v>1727</v>
       </c>
       <c r="H248" t="s">
@@ -14089,7 +14064,7 @@
       <c r="B249" s="27" t="s">
         <v>1992</v>
       </c>
-      <c r="G249" s="81" t="s">
+      <c r="G249" s="82" t="s">
         <v>1727</v>
       </c>
       <c r="H249" t="s">
@@ -14115,7 +14090,7 @@
       <c r="F250" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="G250" s="81" t="s">
+      <c r="G250" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H250" t="s">
@@ -14134,7 +14109,7 @@
       </c>
       <c r="E251" s="3"/>
       <c r="F251" s="3"/>
-      <c r="G251" s="81" t="s">
+      <c r="G251" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H251" t="s">
@@ -14153,7 +14128,7 @@
       </c>
       <c r="E252" s="3"/>
       <c r="F252" s="3"/>
-      <c r="G252" s="81" t="s">
+      <c r="G252" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H252" t="s">
@@ -14179,7 +14154,7 @@
       <c r="F253" s="3" t="s">
         <v>765</v>
       </c>
-      <c r="G253" s="81" t="s">
+      <c r="G253" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H253" t="s">
@@ -14205,7 +14180,7 @@
       <c r="F254" s="3" t="s">
         <v>765</v>
       </c>
-      <c r="G254" s="81" t="s">
+      <c r="G254" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H254" t="s">
@@ -14224,7 +14199,7 @@
       </c>
       <c r="E255" s="76"/>
       <c r="F255" s="3"/>
-      <c r="G255" s="81" t="s">
+      <c r="G255" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H255" t="s">
@@ -14246,7 +14221,7 @@
       </c>
       <c r="E256" s="3"/>
       <c r="F256" s="3"/>
-      <c r="G256" s="81" t="s">
+      <c r="G256" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H256" t="s">
@@ -14256,7 +14231,7 @@
         <v>1964</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A257" s="1" t="s">
         <v>1152</v>
       </c>
@@ -14267,7 +14242,7 @@
       <c r="D257" s="3"/>
       <c r="E257" s="3"/>
       <c r="F257" s="3"/>
-      <c r="G257" s="81" t="s">
+      <c r="G257" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H257" t="s">
@@ -14277,14 +14252,14 @@
         <v>1964</v>
       </c>
     </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A258" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B258" s="30" t="s">
         <v>687</v>
       </c>
-      <c r="G258" s="81" t="s">
+      <c r="G258" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H258" t="s">
@@ -14294,14 +14269,14 @@
         <v>1964</v>
       </c>
     </row>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A259" s="1" t="s">
         <v>1152</v>
       </c>
       <c r="B259" s="30" t="s">
         <v>686</v>
       </c>
-      <c r="G259" s="81" t="s">
+      <c r="G259" s="82" t="s">
         <v>1618</v>
       </c>
       <c r="H259" t="s">
@@ -14311,7 +14286,7 @@
         <v>1964</v>
       </c>
     </row>
-    <row r="260" spans="1:12" s="180" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:11" s="175" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A260" s="1" t="s">
         <v>1152</v>
       </c>
@@ -14326,7 +14301,7 @@
       <c r="F260" t="s">
         <v>766</v>
       </c>
-      <c r="G260" s="81" t="s">
+      <c r="G260" s="182" t="s">
         <v>1619</v>
       </c>
       <c r="H260" t="s">
@@ -14337,203 +14312,196 @@
       </c>
       <c r="J260"/>
     </row>
-    <row r="261" spans="1:12" s="180" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A261" s="187" t="s">
+    <row r="261" spans="1:11" s="175" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A261" s="180" t="s">
         <v>1152</v>
       </c>
-      <c r="B261" s="185" t="s">
+      <c r="B261" s="178" t="s">
         <v>2211</v>
       </c>
-      <c r="C261" s="185"/>
-      <c r="D261" s="185"/>
-      <c r="E261" s="185"/>
-      <c r="F261" s="185"/>
-      <c r="G261" s="188"/>
-      <c r="H261" s="186" t="s">
+      <c r="C261" s="178"/>
+      <c r="D261" s="178"/>
+      <c r="E261" s="178"/>
+      <c r="F261" s="178"/>
+      <c r="G261" s="179" t="s">
         <v>1619</v>
       </c>
-      <c r="I261" s="185" t="s">
+      <c r="H261" s="178" t="s">
         <v>1878</v>
       </c>
-      <c r="J261" s="185" t="s">
+      <c r="I261" s="178" t="s">
         <v>1964</v>
       </c>
-      <c r="K261" s="185">
+      <c r="J261" s="178">
         <v>20260422</v>
       </c>
-      <c r="L261" s="185" t="s">
+      <c r="K261" s="178" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="262" spans="1:12" s="180" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A262" s="187" t="s">
+    <row r="262" spans="1:11" s="175" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A262" s="180" t="s">
         <v>1152</v>
       </c>
-      <c r="B262" s="185" t="s">
+      <c r="B262" s="178" t="s">
         <v>2212</v>
       </c>
-      <c r="C262" s="185"/>
-      <c r="D262" s="185"/>
-      <c r="E262" s="185"/>
-      <c r="F262" s="185"/>
-      <c r="G262" s="188"/>
-      <c r="H262" s="186" t="s">
+      <c r="C262" s="178"/>
+      <c r="D262" s="178"/>
+      <c r="E262" s="178"/>
+      <c r="F262" s="178"/>
+      <c r="G262" s="179" t="s">
         <v>1619</v>
       </c>
-      <c r="I262" s="185" t="s">
+      <c r="H262" s="178" t="s">
         <v>1878</v>
       </c>
-      <c r="J262" s="185" t="s">
+      <c r="I262" s="178" t="s">
         <v>1964</v>
       </c>
-      <c r="K262" s="185">
+      <c r="J262" s="178">
         <v>20260422</v>
       </c>
-      <c r="L262" s="185" t="s">
+      <c r="K262" s="178" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="263" spans="1:12" s="180" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A263" s="187" t="s">
+    <row r="263" spans="1:11" s="175" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A263" s="180" t="s">
         <v>1152</v>
       </c>
-      <c r="B263" s="185" t="s">
+      <c r="B263" s="178" t="s">
         <v>2213</v>
       </c>
-      <c r="C263" s="185"/>
-      <c r="D263" s="185"/>
-      <c r="E263" s="185"/>
-      <c r="F263" s="185"/>
-      <c r="G263" s="188"/>
-      <c r="H263" s="186" t="s">
+      <c r="C263" s="178"/>
+      <c r="D263" s="178"/>
+      <c r="E263" s="178"/>
+      <c r="F263" s="178"/>
+      <c r="G263" s="179" t="s">
         <v>1619</v>
       </c>
-      <c r="I263" s="185" t="s">
+      <c r="H263" s="178" t="s">
         <v>1878</v>
       </c>
-      <c r="J263" s="185" t="s">
+      <c r="I263" s="178" t="s">
         <v>1964</v>
       </c>
-      <c r="K263" s="185">
+      <c r="J263" s="178">
         <v>20260422</v>
       </c>
-      <c r="L263" s="185" t="s">
+      <c r="K263" s="178" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="264" spans="1:12" s="180" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A264" s="187" t="s">
+    <row r="264" spans="1:11" s="175" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A264" s="180" t="s">
         <v>1152</v>
       </c>
-      <c r="B264" s="185" t="s">
+      <c r="B264" s="178" t="s">
         <v>2214</v>
       </c>
-      <c r="C264" s="185"/>
-      <c r="D264" s="185"/>
-      <c r="E264" s="185"/>
-      <c r="F264" s="185"/>
-      <c r="G264" s="188"/>
-      <c r="H264" s="186" t="s">
+      <c r="C264" s="178"/>
+      <c r="D264" s="178"/>
+      <c r="E264" s="178"/>
+      <c r="F264" s="178"/>
+      <c r="G264" s="179" t="s">
         <v>1619</v>
       </c>
-      <c r="I264" s="185" t="s">
+      <c r="H264" s="178" t="s">
         <v>1878</v>
       </c>
-      <c r="J264" s="185" t="s">
+      <c r="I264" s="178" t="s">
         <v>1964</v>
       </c>
-      <c r="K264" s="185">
+      <c r="J264" s="178">
         <v>20260422</v>
       </c>
-      <c r="L264" s="185" t="s">
+      <c r="K264" s="178" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="265" spans="1:12" s="180" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A265" s="187" t="s">
+    <row r="265" spans="1:11" s="175" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A265" s="180" t="s">
         <v>1152</v>
       </c>
-      <c r="B265" s="185" t="s">
+      <c r="B265" s="178" t="s">
         <v>2215</v>
       </c>
-      <c r="C265" s="185"/>
-      <c r="D265" s="185"/>
-      <c r="E265" s="185"/>
-      <c r="F265" s="185"/>
-      <c r="G265" s="188"/>
-      <c r="H265" s="186" t="s">
+      <c r="C265" s="178"/>
+      <c r="D265" s="178"/>
+      <c r="E265" s="178"/>
+      <c r="F265" s="178"/>
+      <c r="G265" s="179" t="s">
         <v>1619</v>
       </c>
-      <c r="I265" s="185" t="s">
+      <c r="H265" s="178" t="s">
         <v>1878</v>
       </c>
-      <c r="J265" s="185" t="s">
+      <c r="I265" s="178" t="s">
         <v>1964</v>
       </c>
-      <c r="K265" s="185">
+      <c r="J265" s="178">
         <v>20260422</v>
       </c>
-      <c r="L265" s="185" t="s">
+      <c r="K265" s="178" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="266" spans="1:12" s="180" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A266" s="187" t="s">
+    <row r="266" spans="1:11" s="175" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A266" s="180" t="s">
         <v>1152</v>
       </c>
-      <c r="B266" s="185" t="s">
+      <c r="B266" s="178" t="s">
         <v>2216</v>
       </c>
-      <c r="C266" s="185"/>
-      <c r="D266" s="185"/>
-      <c r="E266" s="185"/>
-      <c r="F266" s="185"/>
-      <c r="G266" s="188"/>
-      <c r="H266" s="186" t="s">
+      <c r="C266" s="178"/>
+      <c r="D266" s="178"/>
+      <c r="E266" s="178"/>
+      <c r="F266" s="178"/>
+      <c r="G266" s="179" t="s">
         <v>1619</v>
       </c>
-      <c r="I266" s="185" t="s">
+      <c r="H266" s="178" t="s">
         <v>1878</v>
       </c>
-      <c r="J266" s="185" t="s">
+      <c r="I266" s="178" t="s">
         <v>1964</v>
       </c>
-      <c r="K266" s="185">
+      <c r="J266" s="178">
         <v>20260422</v>
       </c>
-      <c r="L266" s="185" t="s">
+      <c r="K266" s="178" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="267" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A267" s="187" t="s">
+    <row r="267" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A267" s="180" t="s">
         <v>1152</v>
       </c>
-      <c r="B267" s="185" t="s">
+      <c r="B267" s="178" t="s">
         <v>2217</v>
       </c>
-      <c r="C267" s="185"/>
-      <c r="D267" s="185"/>
-      <c r="E267" s="185"/>
-      <c r="F267" s="185"/>
-      <c r="G267" s="188"/>
-      <c r="H267" s="186" t="s">
+      <c r="C267" s="178"/>
+      <c r="D267" s="178"/>
+      <c r="E267" s="178"/>
+      <c r="F267" s="178"/>
+      <c r="G267" s="179" t="s">
         <v>1619</v>
       </c>
-      <c r="I267" s="185" t="s">
+      <c r="H267" s="178" t="s">
         <v>1878</v>
       </c>
-      <c r="J267" s="185" t="s">
+      <c r="I267" s="178" t="s">
         <v>1964</v>
       </c>
-      <c r="K267" s="185">
+      <c r="J267" s="178">
         <v>20260422</v>
       </c>
-      <c r="L267" s="185" t="s">
+      <c r="K267" s="178" t="s">
         <v>2173</v>
       </c>
     </row>
-    <row r="268" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A268" s="1" t="s">
         <v>1275</v>
       </c>
@@ -14550,7 +14518,7 @@
         <v>20220909</v>
       </c>
     </row>
-    <row r="269" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A269" s="1" t="s">
         <v>1275</v>
       </c>
@@ -14564,7 +14532,7 @@
         <v>1911</v>
       </c>
     </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A270" s="1" t="s">
         <v>1275</v>
       </c>
@@ -14578,7 +14546,7 @@
         <v>1809</v>
       </c>
     </row>
-    <row r="271" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A271" s="1" t="s">
         <v>1275</v>
       </c>
@@ -14592,7 +14560,7 @@
         <v>1820</v>
       </c>
     </row>
-    <row r="272" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A272" s="1" t="s">
         <v>1275</v>
       </c>

</xml_diff>